<commit_message>
aalterado para usuario consulta
</commit_message>
<xml_diff>
--- a/FLUXO DE CAIXA_labtrans.xlsx
+++ b/FLUXO DE CAIXA_labtrans.xlsx
@@ -2035,7 +2035,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="pt-BR"/>
               </a:p>
@@ -2317,7 +2317,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="pt-BR"/>
               </a:p>
@@ -2445,7 +2445,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="pt-BR"/>
           </a:p>
@@ -2507,7 +2507,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="pt-BR"/>
           </a:p>
@@ -55944,7 +55944,7 @@
         <v>37371852</v>
       </c>
       <c r="D2" s="303" t="n">
-        <v>40809982.36</v>
+        <v>40811325.7</v>
       </c>
       <c r="E2" s="303" t="n">
         <v>27618822.58</v>
@@ -55971,7 +55971,7 @@
         <v>25200000</v>
       </c>
       <c r="D3" s="303" t="n">
-        <v>9628592.369999999</v>
+        <v>9631049.59</v>
       </c>
       <c r="E3" s="303" t="n">
         <v>4604998.83</v>
@@ -56025,7 +56025,7 @@
         <v>1989653</v>
       </c>
       <c r="D5" s="303" t="n">
-        <v>1645041.35</v>
+        <v>1645358.15</v>
       </c>
       <c r="E5" s="303" t="n">
         <v>216680.51</v>
@@ -56052,7 +56052,7 @@
         <v>14412319</v>
       </c>
       <c r="D6" s="303" t="n">
-        <v>19260998.75</v>
+        <v>19322256.47</v>
       </c>
       <c r="E6" s="303" t="n">
         <v>15933478.84</v>
@@ -56703,7 +56703,7 @@
         <v>7</v>
       </c>
       <c r="D31" s="303" t="n">
-        <v>326914.85</v>
+        <v>328201.59</v>
       </c>
       <c r="E31" s="303" t="n">
         <v>46258.11</v>
@@ -57482,7 +57482,7 @@
         <v>7</v>
       </c>
       <c r="D72" s="303" t="n">
-        <v>864626.3100000001</v>
+        <v>925884.03</v>
       </c>
       <c r="E72" s="303" t="n">
         <v>15950</v>

</xml_diff>